<commit_message>
feat: add deadline management and notification system for student group registration
</commit_message>
<xml_diff>
--- a/server/Xep Nhom.xlsx
+++ b/server/Xep Nhom.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\project\exe\jumpln-app-backend-java-spring\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\project\exe\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E171F923-9DBA-4B76-97F5-A72B2BE12A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B04960-4044-4847-8817-2184016F7682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FEA22E60-8B8D-479F-9D0F-795F51FE5A7C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FEA22E60-8B8D-479F-9D0F-795F51FE5A7C}"/>
   </bookViews>
   <sheets>
     <sheet name="EXE101" sheetId="1" r:id="rId1"/>
@@ -46,9 +46,6 @@
   </si>
   <si>
     <t xml:space="preserve">A24/EXE   </t>
-  </si>
-  <si>
-    <t>EXE101_G01</t>
   </si>
   <si>
     <t>Group Mentor</t>
@@ -142,19 +139,22 @@
 *Xếp nhóm </t>
   </si>
   <si>
-    <t>djnd</t>
-  </si>
-  <si>
-    <t>voanhbendjndnd@gmail.com</t>
-  </si>
-  <si>
-    <t>MEMBERCODEEXCEPLE1</t>
-  </si>
-  <si>
-    <t>Duong Nguyen Bao Ngoc</t>
-  </si>
-  <si>
-    <t>CS190012</t>
+    <t>trang</t>
+  </si>
+  <si>
+    <t>EXE101_G02</t>
+  </si>
+  <si>
+    <t>voanhben102@gmail.com</t>
+  </si>
+  <si>
+    <t>LALA</t>
+  </si>
+  <si>
+    <t>CS190014</t>
+  </si>
+  <si>
+    <t>MEMBERCODEEXCEPLE2</t>
   </si>
 </sst>
 </file>
@@ -244,10 +244,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -587,84 +587,84 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" style="1" customWidth="1"/>
     <col min="3" max="3" width="23" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="28.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.44140625" style="1" customWidth="1"/>
     <col min="11" max="11" width="19" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="10.85546875" style="1"/>
+    <col min="12" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+    <row r="1" spans="1:11" ht="88.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
       <c r="K1" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="2" customFormat="1" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>18</v>
       </c>
       <c r="G3" t="s">
@@ -674,10 +674,10 @@
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement deadline management and student group activity features
</commit_message>
<xml_diff>
--- a/server/Xep Nhom.xlsx
+++ b/server/Xep Nhom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\project\exe\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60618624-8C2C-4F33-9421-4D68124B501C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C66B65-373F-46E1-BEC2-83C93644CC1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="23052" yWindow="696" windowWidth="23016" windowHeight="12216" xr2:uid="{FEA22E60-8B8D-479F-9D0F-795F51FE5A7C}"/>
   </bookViews>
@@ -143,9 +143,6 @@
     <t>EXE101_G02</t>
   </si>
   <si>
-    <t>voanhben102@gmail.com</t>
-  </si>
-  <si>
     <t>CS190014</t>
   </si>
   <si>
@@ -171,6 +168,9 @@
   </si>
   <si>
     <t>voanhben103@gmail.com</t>
+  </si>
+  <si>
+    <t>voanhbendjndndnd@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -672,19 +672,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
         <v>2</v>
@@ -696,7 +696,7 @@
         <v>16</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -704,19 +704,19 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>26</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>2</v>
@@ -728,7 +728,7 @@
         <v>16</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>